<commit_message>
Ajustes sección de procesos
</commit_message>
<xml_diff>
--- a/data/raw/Indicadores por CMI.xlsx
+++ b/data/raw/Indicadores por CMI.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Proyectos_DS/Sistema_Indicadores_Poli/data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://poligran-my.sharepoint.com/personal/lxisilva_poligran_edu_co/Documents/Documentos/Proyectos/Sistema_Indicadores_Poli/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="2184" documentId="13_ncr:1_{F0BBE5C6-CAE9-4853-BBB4-310E5D3E7ED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD558F55-0728-4FC4-AE82-EF8F9BC11E43}"/>
@@ -37189,17 +37189,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eb4e1f33-0654-4877-a695-74ac1243131b" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="787dcc16-ad9c-4aed-8595-d8b714944830">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101004B3553A73F55864994CAF6806DB2233B" ma:contentTypeVersion="15" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="0772d54a1d010170e6fbd4301e22082d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="787dcc16-ad9c-4aed-8595-d8b714944830" xmlns:ns3="eb4e1f33-0654-4877-a695-74ac1243131b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d309db89fd7fb813f1d992ce290f04b6" ns2:_="" ns3:_="">
     <xsd:import namespace="787dcc16-ad9c-4aed-8595-d8b714944830"/>
@@ -37434,6 +37423,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eb4e1f33-0654-4877-a695-74ac1243131b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="787dcc16-ad9c-4aed-8595-d8b714944830">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A465C7F-6E2C-46F5-B371-BD23E458BF78}">
   <ds:schemaRefs>
@@ -37443,17 +37443,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F29CE81-ECA4-464A-90AD-CBCC4B67C9CD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="eb4e1f33-0654-4877-a695-74ac1243131b"/>
-    <ds:schemaRef ds:uri="787dcc16-ad9c-4aed-8595-d8b714944830"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0065C2A-D54D-4F3D-A68A-F49590152888}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -37470,4 +37459,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F29CE81-ECA4-464A-90AD-CBCC4B67C9CD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="eb4e1f33-0654-4877-a695-74ac1243131b"/>
+    <ds:schemaRef ds:uri="787dcc16-ad9c-4aed-8595-d8b714944830"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add CMI catalog, new tabs and robustness fixes
Load 'Indicadores por CMI.xlsx' and add UI for CMI catalog: new "Procesos y Unidades", "Indicadores" and "Alertas" tabs, plus heatmap and summary charts. Improve robustness for visualizations: ensure sunburst always receives a fallback row when data or cumplimiento_pct is missing, coerce cumplimiento_pct to numeric, and handle empty objetivo datasets. Extend filters (Unidad, Proceso, Subproceso, Frecuencia, Clasificación, Tipo de indicador) with dependent filtering and segmented controls. Enhance tracking preparation to include Unidad mapping and populate Unidad in output. Add helper functions to load and render CMI catalog summaries and integrate existing alert and heatmap components. Small UI/layout adjustments and defensive checks when files or columns are absent.
</commit_message>
<xml_diff>
--- a/data/raw/Indicadores por CMI.xlsx
+++ b/data/raw/Indicadores por CMI.xlsx
@@ -75770,8 +75770,8 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="A490:A493">
     <cfRule type="duplicateValues" dxfId="94" priority="92"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="94"/>
     <cfRule type="duplicateValues" dxfId="92" priority="93"/>
-    <cfRule type="duplicateValues" dxfId="93" priority="94"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A494">
     <cfRule type="duplicateValues" dxfId="91" priority="85"/>
@@ -75780,34 +75780,34 @@
     <cfRule type="duplicateValues" dxfId="88" priority="89"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A495:A496">
-    <cfRule type="duplicateValues" dxfId="84" priority="79"/>
-    <cfRule type="duplicateValues" dxfId="85" priority="81"/>
     <cfRule type="duplicateValues" dxfId="87" priority="82"/>
     <cfRule type="duplicateValues" dxfId="86" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="81"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="79"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A497:A499">
+    <cfRule type="duplicateValues" dxfId="83" priority="77"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="75"/>
     <cfRule type="duplicateValues" dxfId="80" priority="73"/>
-    <cfRule type="duplicateValues" dxfId="81" priority="75"/>
-    <cfRule type="duplicateValues" dxfId="82" priority="76"/>
-    <cfRule type="duplicateValues" dxfId="83" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A500">
+    <cfRule type="duplicateValues" dxfId="79" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="71"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="70"/>
     <cfRule type="duplicateValues" dxfId="76" priority="67"/>
-    <cfRule type="duplicateValues" dxfId="79" priority="69"/>
-    <cfRule type="duplicateValues" dxfId="77" priority="70"/>
-    <cfRule type="duplicateValues" dxfId="78" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A501:A502">
     <cfRule type="duplicateValues" dxfId="75" priority="61"/>
     <cfRule type="duplicateValues" dxfId="74" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="65"/>
     <cfRule type="duplicateValues" dxfId="72" priority="64"/>
-    <cfRule type="duplicateValues" dxfId="73" priority="65"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A503">
+    <cfRule type="duplicateValues" dxfId="71" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="59"/>
     <cfRule type="duplicateValues" dxfId="69" priority="55"/>
     <cfRule type="duplicateValues" dxfId="68" priority="57"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="58"/>
-    <cfRule type="duplicateValues" dxfId="70" priority="59"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A504:A505">
     <cfRule type="duplicateValues" dxfId="67" priority="49"/>
@@ -75816,22 +75816,22 @@
     <cfRule type="duplicateValues" dxfId="64" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A506">
-    <cfRule type="duplicateValues" dxfId="60" priority="37"/>
     <cfRule type="duplicateValues" dxfId="63" priority="39"/>
     <cfRule type="duplicateValues" dxfId="62" priority="40"/>
     <cfRule type="duplicateValues" dxfId="61" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A507:A508">
     <cfRule type="duplicateValues" dxfId="59" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="46"/>
     <cfRule type="duplicateValues" dxfId="56" priority="45"/>
-    <cfRule type="duplicateValues" dxfId="57" priority="46"/>
-    <cfRule type="duplicateValues" dxfId="58" priority="47"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A509">
+    <cfRule type="duplicateValues" dxfId="55" priority="35"/>
     <cfRule type="duplicateValues" dxfId="54" priority="31"/>
     <cfRule type="duplicateValues" dxfId="53" priority="33"/>
     <cfRule type="duplicateValues" dxfId="52" priority="34"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A510:A578">
     <cfRule type="duplicateValues" dxfId="51" priority="21"/>
@@ -75840,34 +75840,34 @@
     <cfRule type="duplicateValues" dxfId="48" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A579:A580">
-    <cfRule type="duplicateValues" dxfId="44" priority="15"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="17"/>
     <cfRule type="duplicateValues" dxfId="47" priority="18"/>
     <cfRule type="duplicateValues" dxfId="46" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A582:A583">
+    <cfRule type="duplicateValues" dxfId="43" priority="9"/>
     <cfRule type="duplicateValues" dxfId="42" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="43" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="11"/>
     <cfRule type="duplicateValues" dxfId="40" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A585:A592">
-    <cfRule type="duplicateValues" dxfId="36" priority="1"/>
     <cfRule type="duplicateValues" dxfId="39" priority="3"/>
     <cfRule type="duplicateValues" dxfId="38" priority="4"/>
     <cfRule type="duplicateValues" dxfId="37" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B291">
     <cfRule type="duplicateValues" dxfId="35" priority="27"/>
     <cfRule type="duplicateValues" dxfId="34" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B292">
+    <cfRule type="duplicateValues" dxfId="33" priority="30"/>
     <cfRule type="duplicateValues" dxfId="32" priority="29"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B490:B493">
+    <cfRule type="duplicateValues" dxfId="31" priority="95"/>
     <cfRule type="duplicateValues" dxfId="30" priority="91"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="95"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B494">
     <cfRule type="duplicateValues" dxfId="29" priority="86"/>
@@ -75882,28 +75882,28 @@
     <cfRule type="duplicateValues" dxfId="24" priority="78"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B500">
+    <cfRule type="duplicateValues" dxfId="23" priority="72"/>
     <cfRule type="duplicateValues" dxfId="22" priority="68"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="72"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B501:B502">
     <cfRule type="duplicateValues" dxfId="21" priority="62"/>
     <cfRule type="duplicateValues" dxfId="20" priority="66"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B503">
+    <cfRule type="duplicateValues" dxfId="19" priority="60"/>
     <cfRule type="duplicateValues" dxfId="18" priority="56"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="60"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B504:B505">
+    <cfRule type="duplicateValues" dxfId="17" priority="54"/>
     <cfRule type="duplicateValues" dxfId="16" priority="50"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="54"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B506">
     <cfRule type="duplicateValues" dxfId="15" priority="38"/>
     <cfRule type="duplicateValues" dxfId="14" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B507:B508">
+    <cfRule type="duplicateValues" dxfId="13" priority="48"/>
     <cfRule type="duplicateValues" dxfId="12" priority="44"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B509">
     <cfRule type="duplicateValues" dxfId="11" priority="32"/>
@@ -75914,20 +75914,20 @@
     <cfRule type="duplicateValues" dxfId="8" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B579:B580">
+    <cfRule type="duplicateValues" dxfId="7" priority="20"/>
     <cfRule type="duplicateValues" dxfId="6" priority="16"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B581">
+    <cfRule type="duplicateValues" dxfId="5" priority="14"/>
     <cfRule type="duplicateValues" dxfId="4" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B582:B583">
+    <cfRule type="duplicateValues" dxfId="3" priority="12"/>
     <cfRule type="duplicateValues" dxfId="2" priority="8"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B585:B592">
+    <cfRule type="duplicateValues" dxfId="1" priority="6"/>
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="6"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -76780,15 +76780,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101004B3553A73F55864994CAF6806DB2233B" ma:contentTypeVersion="15" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="0772d54a1d010170e6fbd4301e22082d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="787dcc16-ad9c-4aed-8595-d8b714944830" xmlns:ns3="eb4e1f33-0654-4877-a695-74ac1243131b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d309db89fd7fb813f1d992ce290f04b6" ns2:_="" ns3:_="">
     <xsd:import namespace="787dcc16-ad9c-4aed-8595-d8b714944830"/>
@@ -77023,6 +77014,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -77035,14 +77035,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A465C7F-6E2C-46F5-B371-BD23E458BF78}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0065C2A-D54D-4F3D-A68A-F49590152888}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -77061,6 +77053,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A465C7F-6E2C-46F5-B371-BD23E458BF78}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F29CE81-ECA4-464A-90AD-CBCC4B67C9CD}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Revert "Ajustes sección de procesos"
This reverts commit 1fece2b5bbaa9b62e896830ff1ab8dbd49497c5e.
</commit_message>
<xml_diff>
--- a/data/raw/Indicadores por CMI.xlsx
+++ b/data/raw/Indicadores por CMI.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://poligran-my.sharepoint.com/personal/lxisilva_poligran_edu_co/Documents/Documentos/Proyectos/Sistema_Indicadores_Poli/data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Proyectos_DS/Sistema_Indicadores_Poli/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2495" documentId="13_ncr:1_{F0BBE5C6-CAE9-4853-BBB4-310E5D3E7ED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3379351E-04EE-4600-BF73-76FBA0887C84}"/>
+  <xr:revisionPtr revIDLastSave="2475" documentId="13_ncr:1_{F0BBE5C6-CAE9-4853-BBB4-310E5D3E7ED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7712E354-5FB0-4F59-A7B6-34EF38AD806A}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-705" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -27574,9 +27574,7 @@
         <v>1</v>
       </c>
       <c r="N351" s="4"/>
-      <c r="O351" s="4">
-        <v>0</v>
-      </c>
+      <c r="O351" s="4"/>
       <c r="P351" s="4"/>
       <c r="Q351" s="4">
         <v>1</v>
@@ -27639,9 +27637,7 @@
         <v>1</v>
       </c>
       <c r="N352" s="4"/>
-      <c r="O352" s="4">
-        <v>0</v>
-      </c>
+      <c r="O352" s="4"/>
       <c r="P352" s="4"/>
       <c r="Q352" s="4">
         <v>1</v>
@@ -27704,9 +27700,7 @@
         <v>1</v>
       </c>
       <c r="N353" s="4"/>
-      <c r="O353" s="4">
-        <v>0</v>
-      </c>
+      <c r="O353" s="4"/>
       <c r="P353" s="4"/>
       <c r="Q353" s="4">
         <v>1</v>
@@ -27769,9 +27763,7 @@
         <v>1</v>
       </c>
       <c r="N354" s="4"/>
-      <c r="O354" s="4">
-        <v>0</v>
-      </c>
+      <c r="O354" s="4"/>
       <c r="P354" s="4"/>
       <c r="Q354" s="4">
         <v>1</v>
@@ -27834,9 +27826,7 @@
         <v>1</v>
       </c>
       <c r="N355" s="4"/>
-      <c r="O355" s="4">
-        <v>0</v>
-      </c>
+      <c r="O355" s="4"/>
       <c r="P355" s="4"/>
       <c r="Q355" s="4">
         <v>1</v>
@@ -27899,9 +27889,7 @@
         <v>1</v>
       </c>
       <c r="N356" s="4"/>
-      <c r="O356" s="4">
-        <v>0</v>
-      </c>
+      <c r="O356" s="4"/>
       <c r="P356" s="4"/>
       <c r="Q356" s="4">
         <v>1</v>
@@ -27964,9 +27952,7 @@
         <v>1</v>
       </c>
       <c r="N357" s="4"/>
-      <c r="O357" s="4">
-        <v>0</v>
-      </c>
+      <c r="O357" s="4"/>
       <c r="P357" s="4"/>
       <c r="Q357" s="4">
         <v>1</v>
@@ -29428,9 +29414,7 @@
       <c r="L381" s="4"/>
       <c r="M381" s="4"/>
       <c r="N381" s="4"/>
-      <c r="O381" s="4">
-        <v>0</v>
-      </c>
+      <c r="O381" s="4"/>
       <c r="P381" s="4"/>
       <c r="Q381" s="4">
         <v>1</v>
@@ -36055,9 +36039,7 @@
       <c r="L490" s="4"/>
       <c r="M490" s="4"/>
       <c r="N490" s="4"/>
-      <c r="O490" s="4">
-        <v>0</v>
-      </c>
+      <c r="O490" s="4"/>
       <c r="P490" s="4"/>
       <c r="Q490" s="4"/>
       <c r="R490" s="4"/>
@@ -36110,9 +36092,7 @@
       <c r="L491" s="4"/>
       <c r="M491" s="4"/>
       <c r="N491" s="4"/>
-      <c r="O491" s="4">
-        <v>0</v>
-      </c>
+      <c r="O491" s="4"/>
       <c r="P491" s="4"/>
       <c r="Q491" s="4"/>
       <c r="R491" s="4"/>
@@ -36165,9 +36145,7 @@
       <c r="L492" s="4"/>
       <c r="M492" s="4"/>
       <c r="N492" s="4"/>
-      <c r="O492" s="4">
-        <v>0</v>
-      </c>
+      <c r="O492" s="4"/>
       <c r="P492" s="4"/>
       <c r="Q492" s="4"/>
       <c r="R492" s="4"/>
@@ -36220,9 +36198,7 @@
       <c r="L493" s="4"/>
       <c r="M493" s="4"/>
       <c r="N493" s="4"/>
-      <c r="O493" s="4">
-        <v>0</v>
-      </c>
+      <c r="O493" s="4"/>
       <c r="P493" s="4"/>
       <c r="Q493" s="4"/>
       <c r="R493" s="4"/>
@@ -41782,7 +41758,6 @@
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
-  <autoFilter ref="A1:W595" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="A109">
     <cfRule type="duplicateValues" dxfId="213" priority="113"/>
   </conditionalFormatting>
@@ -76805,14 +76780,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eb4e1f33-0654-4877-a695-74ac1243131b" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="787dcc16-ad9c-4aed-8595-d8b714944830">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -77051,21 +77024,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eb4e1f33-0654-4877-a695-74ac1243131b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="787dcc16-ad9c-4aed-8595-d8b714944830">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F29CE81-ECA4-464A-90AD-CBCC4B67C9CD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A465C7F-6E2C-46F5-B371-BD23E458BF78}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="eb4e1f33-0654-4877-a695-74ac1243131b"/>
-    <ds:schemaRef ds:uri="787dcc16-ad9c-4aed-8595-d8b714944830"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -77090,9 +77062,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A465C7F-6E2C-46F5-B371-BD23E458BF78}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F29CE81-ECA4-464A-90AD-CBCC4B67C9CD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="eb4e1f33-0654-4877-a695-74ac1243131b"/>
+    <ds:schemaRef ds:uri="787dcc16-ad9c-4aed-8595-d8b714944830"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>